<commit_message>
Corrida | SFE-EIP | 2026-06-17 11:52:08.141875
</commit_message>
<xml_diff>
--- a/indicadores/SFE-EIP_out.xlsx
+++ b/indicadores/SFE-EIP_out.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="536" uniqueCount="536">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="538" uniqueCount="538">
   <si>
     <t xml:space="preserve"/>
   </si>
@@ -74,6 +74,12 @@
     <t xml:space="preserve">td1coef</t>
   </si>
   <si>
+    <t xml:space="preserve">Alcance</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Provincia de Santa Fe</t>
+  </si>
+  <si>
     <t xml:space="preserve">Resumen del correlograma</t>
   </si>
   <si>
@@ -107,13 +113,13 @@
     <t xml:space="preserve">Fecha</t>
   </si>
   <si>
-    <t xml:space="preserve">27/05/2026</t>
+    <t xml:space="preserve">17/06/2026</t>
   </si>
   <si>
     <t xml:space="preserve">Usuario</t>
   </si>
   <si>
-    <t xml:space="preserve">arodriguez</t>
+    <t xml:space="preserve">focampo</t>
   </si>
   <si>
     <t xml:space="preserve">fecha</t>
@@ -2124,9 +2130,13 @@
       <c r="J6" s="1"/>
     </row>
     <row r="7">
-      <c r="A7"/>
+      <c r="A7" t="s">
+        <v>19</v>
+      </c>
       <c r="B7"/>
-      <c r="C7"/>
+      <c r="C7" t="s">
+        <v>20</v>
+      </c>
       <c r="D7"/>
       <c r="E7"/>
       <c r="F7"/>
@@ -2137,7 +2147,7 @@
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="B8"/>
       <c r="C8"/>
@@ -2151,12 +2161,12 @@
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B9"/>
       <c r="C9"/>
       <c r="D9" t="n">
-        <v>0.52098946735509</v>
+        <v>0.521586057839713</v>
       </c>
       <c r="E9"/>
       <c r="F9"/>
@@ -2167,7 +2177,7 @@
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="B10"/>
       <c r="C10"/>
@@ -2195,7 +2205,7 @@
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B12"/>
       <c r="C12"/>
@@ -2209,12 +2219,12 @@
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="B13"/>
       <c r="C13"/>
       <c r="D13" t="n">
-        <v>0.243226801534299</v>
+        <v>0.244518193107434</v>
       </c>
       <c r="E13"/>
       <c r="F13"/>
@@ -2237,7 +2247,7 @@
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="B15"/>
       <c r="C15"/>
@@ -2251,7 +2261,7 @@
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="B16"/>
       <c r="C16"/>
@@ -2265,7 +2275,7 @@
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="B17"/>
       <c r="C17"/>
@@ -2279,12 +2289,12 @@
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="B18"/>
       <c r="C18"/>
       <c r="D18" t="n">
-        <v>0.00237465496094546</v>
+        <v>0.00277534947348472</v>
       </c>
       <c r="E18"/>
       <c r="F18"/>
@@ -2295,7 +2305,7 @@
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="B19"/>
       <c r="C19"/>
@@ -2309,12 +2319,12 @@
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="B20"/>
       <c r="C20"/>
       <c r="D20" t="n">
-        <v>0.0723099642468708</v>
+        <v>0.0619404959737314</v>
       </c>
       <c r="E20"/>
       <c r="F20"/>
@@ -2457,10 +2467,10 @@
     </row>
     <row r="32">
       <c r="A32" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="B32" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="C32"/>
       <c r="D32"/>
@@ -2473,10 +2483,10 @@
     </row>
     <row r="33">
       <c r="A33" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="B33" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="C33"/>
       <c r="D33"/>
@@ -2500,66 +2510,66 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="B1" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="C1" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="D1" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="E1" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="F1" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="G1" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="H1" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="I1" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="J1" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="K1" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="L1" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="M1" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="N1" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="O1" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="P1" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="Q1" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="R1" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="S1" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="B2" s="2" t="n">
         <v>104.045689417212</v>
@@ -2612,7 +2622,7 @@
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="B3" s="2" t="n">
         <v>105.731882296344</v>
@@ -2669,7 +2679,7 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="B4" s="2" t="n">
         <v>123.478217763771</v>
@@ -2726,7 +2736,7 @@
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="B5" s="2" t="n">
         <v>147.715122616819</v>
@@ -2783,7 +2793,7 @@
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="B6" s="2" t="n">
         <v>161.873371550932</v>
@@ -2840,7 +2850,7 @@
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="B7" s="2" t="n">
         <v>156.884307193375</v>
@@ -2897,7 +2907,7 @@
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="B8" s="2" t="n">
         <v>154.430178964142</v>
@@ -2954,7 +2964,7 @@
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="B9" s="2" t="n">
         <v>150.303525865356</v>
@@ -3011,7 +3021,7 @@
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="B10" s="2" t="n">
         <v>148.489903485932</v>
@@ -3068,7 +3078,7 @@
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="B11" s="2" t="n">
         <v>145.593597529018</v>
@@ -3125,7 +3135,7 @@
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="B12" s="2" t="n">
         <v>133.106931655834</v>
@@ -3182,7 +3192,7 @@
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="B13" s="2" t="n">
         <v>114.542274659608</v>
@@ -3239,7 +3249,7 @@
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="B14" s="2" t="n">
         <v>112.844303500924</v>
@@ -3298,7 +3308,7 @@
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="B15" s="2" t="n">
         <v>111.82570168793</v>
@@ -3357,7 +3367,7 @@
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="B16" s="2" t="n">
         <v>128.788894304159</v>
@@ -3416,7 +3426,7 @@
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="B17" s="2" t="n">
         <v>154.075209779165</v>
@@ -3475,7 +3485,7 @@
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="B18" s="2" t="n">
         <v>162.688373481389</v>
@@ -3534,7 +3544,7 @@
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="B19" s="2" t="n">
         <v>154.841811965375</v>
@@ -3593,7 +3603,7 @@
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="B20" s="2" t="n">
         <v>156.91724447214</v>
@@ -3652,7 +3662,7 @@
     </row>
     <row r="21">
       <c r="A21" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="B21" s="2" t="n">
         <v>153.498918432074</v>
@@ -3711,7 +3721,7 @@
     </row>
     <row r="22">
       <c r="A22" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="B22" s="2" t="n">
         <v>149.558188135168</v>
@@ -3770,7 +3780,7 @@
     </row>
     <row r="23">
       <c r="A23" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="B23" s="2" t="n">
         <v>146.631220152149</v>
@@ -3829,7 +3839,7 @@
     </row>
     <row r="24">
       <c r="A24" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="B24" s="2" t="n">
         <v>134.421009913652</v>
@@ -3888,7 +3898,7 @@
     </row>
     <row r="25">
       <c r="A25" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="B25" s="2" t="n">
         <v>116.300379294692</v>
@@ -3947,7 +3957,7 @@
     </row>
     <row r="26">
       <c r="A26" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B26" s="2" t="n">
         <v>115.157870229313</v>
@@ -4006,7 +4016,7 @@
     </row>
     <row r="27">
       <c r="A27" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="B27" s="2" t="n">
         <v>117.581657991359</v>
@@ -4065,7 +4075,7 @@
     </row>
     <row r="28">
       <c r="A28" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="B28" s="2" t="n">
         <v>139.0641731739</v>
@@ -4124,7 +4134,7 @@
     </row>
     <row r="29">
       <c r="A29" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="B29" s="2" t="n">
         <v>165.177785529658</v>
@@ -4183,7 +4193,7 @@
     </row>
     <row r="30">
       <c r="A30" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="B30" s="2" t="n">
         <v>177.335527240012</v>
@@ -4242,7 +4252,7 @@
     </row>
     <row r="31">
       <c r="A31" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="B31" s="2" t="n">
         <v>171.375388083804</v>
@@ -4301,7 +4311,7 @@
     </row>
     <row r="32">
       <c r="A32" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="B32" s="2" t="n">
         <v>168.802011956629</v>
@@ -4360,7 +4370,7 @@
     </row>
     <row r="33">
       <c r="A33" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="B33" s="2" t="n">
         <v>162.162791630945</v>
@@ -4419,7 +4429,7 @@
     </row>
     <row r="34">
       <c r="A34" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="B34" s="2" t="n">
         <v>162.817363645596</v>
@@ -4478,7 +4488,7 @@
     </row>
     <row r="35">
       <c r="A35" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="B35" s="2" t="n">
         <v>165.563997769355</v>
@@ -4537,7 +4547,7 @@
     </row>
     <row r="36">
       <c r="A36" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="B36" s="2" t="n">
         <v>151.823279287318</v>
@@ -4596,7 +4606,7 @@
     </row>
     <row r="37">
       <c r="A37" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="B37" s="2" t="n">
         <v>128.875487722838</v>
@@ -4655,7 +4665,7 @@
     </row>
     <row r="38">
       <c r="A38" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="B38" s="2" t="n">
         <v>126.679204543358</v>
@@ -4714,7 +4724,7 @@
     </row>
     <row r="39">
       <c r="A39" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="B39" s="2" t="n">
         <v>127.338364840736</v>
@@ -4773,7 +4783,7 @@
     </row>
     <row r="40">
       <c r="A40" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="B40" s="2" t="n">
         <v>146.937550294317</v>
@@ -4832,7 +4842,7 @@
     </row>
     <row r="41">
       <c r="A41" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="B41" s="2" t="n">
         <v>172.351573782611</v>
@@ -4891,7 +4901,7 @@
     </row>
     <row r="42">
       <c r="A42" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="B42" s="2" t="n">
         <v>180.661905849067</v>
@@ -4950,7 +4960,7 @@
     </row>
     <row r="43">
       <c r="A43" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="B43" s="2" t="n">
         <v>169.080642236465</v>
@@ -5009,7 +5019,7 @@
     </row>
     <row r="44">
       <c r="A44" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="B44" s="2" t="n">
         <v>165.021195405505</v>
@@ -5068,7 +5078,7 @@
     </row>
     <row r="45">
       <c r="A45" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="B45" s="2" t="n">
         <v>159.01193649041</v>
@@ -5127,7 +5137,7 @@
     </row>
     <row r="46">
       <c r="A46" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="B46" s="2" t="n">
         <v>157.290545420119</v>
@@ -5186,7 +5196,7 @@
     </row>
     <row r="47">
       <c r="A47" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="B47" s="2" t="n">
         <v>157.95439883404</v>
@@ -5245,7 +5255,7 @@
     </row>
     <row r="48">
       <c r="A48" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="B48" s="2" t="n">
         <v>145.224230904012</v>
@@ -5304,7 +5314,7 @@
     </row>
     <row r="49">
       <c r="A49" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="B49" s="2" t="n">
         <v>124.134697389964</v>
@@ -5363,7 +5373,7 @@
     </row>
     <row r="50">
       <c r="A50" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="B50" s="2" t="n">
         <v>123.302304450303</v>
@@ -5422,7 +5432,7 @@
     </row>
     <row r="51">
       <c r="A51" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="B51" s="2" t="n">
         <v>125.019386234882</v>
@@ -5481,7 +5491,7 @@
     </row>
     <row r="52">
       <c r="A52" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="B52" s="2" t="n">
         <v>147.335567954372</v>
@@ -5540,7 +5550,7 @@
     </row>
     <row r="53">
       <c r="A53" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="B53" s="2" t="n">
         <v>178.627453681345</v>
@@ -5599,7 +5609,7 @@
     </row>
     <row r="54">
       <c r="A54" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="B54" s="2" t="n">
         <v>192.533487871493</v>
@@ -5658,7 +5668,7 @@
     </row>
     <row r="55">
       <c r="A55" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="B55" s="2" t="n">
         <v>184.426440758095</v>
@@ -5717,7 +5727,7 @@
     </row>
     <row r="56">
       <c r="A56" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="B56" s="2" t="n">
         <v>185.362852050619</v>
@@ -5776,7 +5786,7 @@
     </row>
     <row r="57">
       <c r="A57" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="B57" s="2" t="n">
         <v>184.458375505643</v>
@@ -5835,7 +5845,7 @@
     </row>
     <row r="58">
       <c r="A58" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="B58" s="2" t="n">
         <v>184.246780157573</v>
@@ -5894,7 +5904,7 @@
     </row>
     <row r="59">
       <c r="A59" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="B59" s="2" t="n">
         <v>181.8553743494</v>
@@ -5953,7 +5963,7 @@
     </row>
     <row r="60">
       <c r="A60" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="B60" s="2" t="n">
         <v>165.150812818626</v>
@@ -6012,7 +6022,7 @@
     </row>
     <row r="61">
       <c r="A61" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="B61" s="2" t="n">
         <v>139.8806132667</v>
@@ -6071,7 +6081,7 @@
     </row>
     <row r="62">
       <c r="A62" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="B62" s="2" t="n">
         <v>136.973041260878</v>
@@ -6130,7 +6140,7 @@
     </row>
     <row r="63">
       <c r="A63" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="B63" s="2" t="n">
         <v>138.853351946874</v>
@@ -6189,7 +6199,7 @@
     </row>
     <row r="64">
       <c r="A64" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="B64" s="2" t="n">
         <v>162.557385090182</v>
@@ -6248,7 +6258,7 @@
     </row>
     <row r="65">
       <c r="A65" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="B65" s="2" t="n">
         <v>194.652238473962</v>
@@ -6307,7 +6317,7 @@
     </row>
     <row r="66">
       <c r="A66" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="B66" s="2" t="n">
         <v>211.256785041694</v>
@@ -6366,7 +6376,7 @@
     </row>
     <row r="67">
       <c r="A67" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="B67" s="2" t="n">
         <v>205.460689687835</v>
@@ -6425,7 +6435,7 @@
     </row>
     <row r="68">
       <c r="A68" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="B68" s="2" t="n">
         <v>205.173950830816</v>
@@ -6484,7 +6494,7 @@
     </row>
     <row r="69">
       <c r="A69" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="B69" s="2" t="n">
         <v>196.958843573021</v>
@@ -6543,7 +6553,7 @@
     </row>
     <row r="70">
       <c r="A70" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="B70" s="2" t="n">
         <v>192.412637996892</v>
@@ -6602,7 +6612,7 @@
     </row>
     <row r="71">
       <c r="A71" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="B71" s="2" t="n">
         <v>189.639603318676</v>
@@ -6661,7 +6671,7 @@
     </row>
     <row r="72">
       <c r="A72" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="B72" s="2" t="n">
         <v>171.598164071965</v>
@@ -6720,7 +6730,7 @@
     </row>
     <row r="73">
       <c r="A73" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="B73" s="2" t="n">
         <v>147.501322417106</v>
@@ -6779,7 +6789,7 @@
     </row>
     <row r="74">
       <c r="A74" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="B74" s="2" t="n">
         <v>146.336049118133</v>
@@ -6838,7 +6848,7 @@
     </row>
     <row r="75">
       <c r="A75" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="B75" s="2" t="n">
         <v>146.213569925788</v>
@@ -6897,7 +6907,7 @@
     </row>
     <row r="76">
       <c r="A76" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="B76" s="2" t="n">
         <v>170.289189619032</v>
@@ -6956,7 +6966,7 @@
     </row>
     <row r="77">
       <c r="A77" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="B77" s="2" t="n">
         <v>202.506457492855</v>
@@ -7015,7 +7025,7 @@
     </row>
     <row r="78">
       <c r="A78" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="B78" s="2" t="n">
         <v>211.902612739198</v>
@@ -7074,7 +7084,7 @@
     </row>
     <row r="79">
       <c r="A79" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="B79" s="2" t="n">
         <v>199.162167529478</v>
@@ -7133,7 +7143,7 @@
     </row>
     <row r="80">
       <c r="A80" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="B80" s="2" t="n">
         <v>196.954328902439</v>
@@ -7192,7 +7202,7 @@
     </row>
     <row r="81">
       <c r="A81" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="B81" s="2" t="n">
         <v>190.32600903884</v>
@@ -7251,7 +7261,7 @@
     </row>
     <row r="82">
       <c r="A82" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="B82" s="2" t="n">
         <v>186.40362488269</v>
@@ -7310,7 +7320,7 @@
     </row>
     <row r="83">
       <c r="A83" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="B83" s="2" t="n">
         <v>183.118173531313</v>
@@ -7369,7 +7379,7 @@
     </row>
     <row r="84">
       <c r="A84" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="B84" s="2" t="n">
         <v>165.302106600313</v>
@@ -7428,7 +7438,7 @@
     </row>
     <row r="85">
       <c r="A85" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="B85" s="2" t="n">
         <v>140.429163914044</v>
@@ -7487,7 +7497,7 @@
     </row>
     <row r="86">
       <c r="A86" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="B86" s="2" t="n">
         <v>139.131343077671</v>
@@ -7546,7 +7556,7 @@
     </row>
     <row r="87">
       <c r="A87" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="B87" s="2" t="n">
         <v>140.789545428529</v>
@@ -7605,7 +7615,7 @@
     </row>
     <row r="88">
       <c r="A88" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="B88" s="2" t="n">
         <v>164.086368788233</v>
@@ -7664,7 +7674,7 @@
     </row>
     <row r="89">
       <c r="A89" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="B89" s="2" t="n">
         <v>194.975878540515</v>
@@ -7723,7 +7733,7 @@
     </row>
     <row r="90">
       <c r="A90" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="B90" s="2" t="n">
         <v>205.734001320228</v>
@@ -7782,7 +7792,7 @@
     </row>
     <row r="91">
       <c r="A91" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="B91" s="2" t="n">
         <v>193.659697274293</v>
@@ -7841,7 +7851,7 @@
     </row>
     <row r="92">
       <c r="A92" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="B92" s="2" t="n">
         <v>187.247147966469</v>
@@ -7900,7 +7910,7 @@
     </row>
     <row r="93">
       <c r="A93" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="B93" s="2" t="n">
         <v>176.956018319687</v>
@@ -7959,7 +7969,7 @@
     </row>
     <row r="94">
       <c r="A94" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="B94" s="2" t="n">
         <v>172.927589544154</v>
@@ -8018,7 +8028,7 @@
     </row>
     <row r="95">
       <c r="A95" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="B95" s="2" t="n">
         <v>168.121175661017</v>
@@ -8077,7 +8087,7 @@
     </row>
     <row r="96">
       <c r="A96" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="B96" s="2" t="n">
         <v>149.602698179801</v>
@@ -8136,7 +8146,7 @@
     </row>
     <row r="97">
       <c r="A97" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="B97" s="2" t="n">
         <v>125.319583471635</v>
@@ -8195,7 +8205,7 @@
     </row>
     <row r="98">
       <c r="A98" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="B98" s="2" t="n">
         <v>121.144941828202</v>
@@ -8254,7 +8264,7 @@
     </row>
     <row r="99">
       <c r="A99" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="B99" s="2" t="n">
         <v>121.711464059326</v>
@@ -8313,7 +8323,7 @@
     </row>
     <row r="100">
       <c r="A100" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="B100" s="2" t="n">
         <v>142.767753888209</v>
@@ -8372,7 +8382,7 @@
     </row>
     <row r="101">
       <c r="A101" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="B101" s="2" t="n">
         <v>168.468590690473</v>
@@ -8431,7 +8441,7 @@
     </row>
     <row r="102">
       <c r="A102" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="B102" s="2" t="n">
         <v>179.306204204518</v>
@@ -8490,7 +8500,7 @@
     </row>
     <row r="103">
       <c r="A103" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="B103" s="2" t="n">
         <v>172.502271744492</v>
@@ -8549,7 +8559,7 @@
     </row>
     <row r="104">
       <c r="A104" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="B104" s="2" t="n">
         <v>171.618457773098</v>
@@ -8608,7 +8618,7 @@
     </row>
     <row r="105">
       <c r="A105" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="B105" s="2" t="n">
         <v>168.626198392427</v>
@@ -8667,7 +8677,7 @@
     </row>
     <row r="106">
       <c r="A106" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="B106" s="2" t="n">
         <v>169.068525284773</v>
@@ -8726,7 +8736,7 @@
     </row>
     <row r="107">
       <c r="A107" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="B107" s="2" t="n">
         <v>170.711505827028</v>
@@ -8785,7 +8795,7 @@
     </row>
     <row r="108">
       <c r="A108" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="B108" s="2" t="n">
         <v>157.348508232077</v>
@@ -8844,7 +8854,7 @@
     </row>
     <row r="109">
       <c r="A109" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="B109" s="2" t="n">
         <v>132.865288601437</v>
@@ -8903,7 +8913,7 @@
     </row>
     <row r="110">
       <c r="A110" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="B110" s="2" t="n">
         <v>131.038861096426</v>
@@ -8962,7 +8972,7 @@
     </row>
     <row r="111">
       <c r="A111" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="B111" s="2" t="n">
         <v>134.33315633328</v>
@@ -9021,7 +9031,7 @@
     </row>
     <row r="112">
       <c r="A112" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="B112" s="2" t="n">
         <v>156.027712207464</v>
@@ -9080,7 +9090,7 @@
     </row>
     <row r="113">
       <c r="A113" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="B113" s="2" t="n">
         <v>185.636748713923</v>
@@ -9139,7 +9149,7 @@
     </row>
     <row r="114">
       <c r="A114" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="B114" s="2" t="n">
         <v>201.295320593742</v>
@@ -9198,7 +9208,7 @@
     </row>
     <row r="115">
       <c r="A115" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="B115" s="2" t="n">
         <v>193.331665178712</v>
@@ -9257,7 +9267,7 @@
     </row>
     <row r="116">
       <c r="A116" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="B116" s="2" t="n">
         <v>194.590983014024</v>
@@ -9316,7 +9326,7 @@
     </row>
     <row r="117">
       <c r="A117" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="B117" s="2" t="n">
         <v>193.792097074925</v>
@@ -9375,7 +9385,7 @@
     </row>
     <row r="118">
       <c r="A118" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="B118" s="2" t="n">
         <v>195.963660988877</v>
@@ -9434,7 +9444,7 @@
     </row>
     <row r="119">
       <c r="A119" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="B119" s="2" t="n">
         <v>199.743408653628</v>
@@ -9493,7 +9503,7 @@
     </row>
     <row r="120">
       <c r="A120" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="B120" s="2" t="n">
         <v>183.022290796016</v>
@@ -9552,7 +9562,7 @@
     </row>
     <row r="121">
       <c r="A121" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="B121" s="2" t="n">
         <v>154.809191723975</v>
@@ -9611,7 +9621,7 @@
     </row>
     <row r="122">
       <c r="A122" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="B122" s="2" t="n">
         <v>153.813345760426</v>
@@ -9670,7 +9680,7 @@
     </row>
     <row r="123">
       <c r="A123" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="B123" s="2" t="n">
         <v>155.318869927241</v>
@@ -9729,7 +9739,7 @@
     </row>
     <row r="124">
       <c r="A124" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="B124" s="2" t="n">
         <v>179.149156272744</v>
@@ -9788,7 +9798,7 @@
     </row>
     <row r="125">
       <c r="A125" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="B125" s="2" t="n">
         <v>212.083524875889</v>
@@ -9847,7 +9857,7 @@
     </row>
     <row r="126">
       <c r="A126" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="B126" s="2" t="n">
         <v>227.253388339372</v>
@@ -9906,7 +9916,7 @@
     </row>
     <row r="127">
       <c r="A127" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="B127" s="2" t="n">
         <v>218.731317716766</v>
@@ -9965,7 +9975,7 @@
     </row>
     <row r="128">
       <c r="A128" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="B128" s="2" t="n">
         <v>217.07351346441</v>
@@ -10024,7 +10034,7 @@
     </row>
     <row r="129">
       <c r="A129" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="B129" s="2" t="n">
         <v>209.422760217189</v>
@@ -10083,7 +10093,7 @@
     </row>
     <row r="130">
       <c r="A130" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="B130" s="2" t="n">
         <v>206.179154403573</v>
@@ -10142,7 +10152,7 @@
     </row>
     <row r="131">
       <c r="A131" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="B131" s="2" t="n">
         <v>205.138113371857</v>
@@ -10201,7 +10211,7 @@
     </row>
     <row r="132">
       <c r="A132" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="B132" s="2" t="n">
         <v>189.027425582472</v>
@@ -10260,7 +10270,7 @@
     </row>
     <row r="133">
       <c r="A133" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="B133" s="2" t="n">
         <v>165.152771286566</v>
@@ -10319,7 +10329,7 @@
     </row>
     <row r="134">
       <c r="A134" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="B134" s="2" t="n">
         <v>165.700624951205</v>
@@ -10378,7 +10388,7 @@
     </row>
     <row r="135">
       <c r="A135" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="B135" s="2" t="n">
         <v>167.023054546816</v>
@@ -10437,7 +10447,7 @@
     </row>
     <row r="136">
       <c r="A136" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="B136" s="2" t="n">
         <v>194.846321447175</v>
@@ -10496,7 +10506,7 @@
     </row>
     <row r="137">
       <c r="A137" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="B137" s="2" t="n">
         <v>231.563217378506</v>
@@ -10555,7 +10565,7 @@
     </row>
     <row r="138">
       <c r="A138" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="B138" s="2" t="n">
         <v>244.275587445363</v>
@@ -10614,7 +10624,7 @@
     </row>
     <row r="139">
       <c r="A139" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="B139" s="2" t="n">
         <v>232.003321990784</v>
@@ -10673,7 +10683,7 @@
     </row>
     <row r="140">
       <c r="A140" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="B140" s="2" t="n">
         <v>228.981514611917</v>
@@ -10732,7 +10742,7 @@
     </row>
     <row r="141">
       <c r="A141" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="B141" s="2" t="n">
         <v>219.273215690265</v>
@@ -10791,7 +10801,7 @@
     </row>
     <row r="142">
       <c r="A142" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="B142" s="2" t="n">
         <v>214.999111754504</v>
@@ -10850,7 +10860,7 @@
     </row>
     <row r="143">
       <c r="A143" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="B143" s="2" t="n">
         <v>214.196387660624</v>
@@ -10909,7 +10919,7 @@
     </row>
     <row r="144">
       <c r="A144" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="B144" s="2" t="n">
         <v>197.887260471173</v>
@@ -10968,7 +10978,7 @@
     </row>
     <row r="145">
       <c r="A145" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="B145" s="2" t="n">
         <v>171.01790241034</v>
@@ -11027,7 +11037,7 @@
     </row>
     <row r="146">
       <c r="A146" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="B146" s="2" t="n">
         <v>169.92186377084</v>
@@ -11086,7 +11096,7 @@
     </row>
     <row r="147">
       <c r="A147" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="B147" s="2" t="n">
         <v>171.349748496745</v>
@@ -11145,7 +11155,7 @@
     </row>
     <row r="148">
       <c r="A148" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="B148" s="2" t="n">
         <v>198.401889778151</v>
@@ -11204,7 +11214,7 @@
     </row>
     <row r="149">
       <c r="A149" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="B149" s="2" t="n">
         <v>236.383566478328</v>
@@ -11263,7 +11273,7 @@
     </row>
     <row r="150">
       <c r="A150" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="B150" s="2" t="n">
         <v>252.492131180424</v>
@@ -11322,7 +11332,7 @@
     </row>
     <row r="151">
       <c r="A151" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="B151" s="2" t="n">
         <v>242.26156772761</v>
@@ -11381,7 +11391,7 @@
     </row>
     <row r="152">
       <c r="A152" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="B152" s="2" t="n">
         <v>246.468786594478</v>
@@ -11440,7 +11450,7 @@
     </row>
     <row r="153">
       <c r="A153" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="B153" s="2" t="n">
         <v>246.472230270109</v>
@@ -11499,7 +11509,7 @@
     </row>
     <row r="154">
       <c r="A154" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="B154" s="2" t="n">
         <v>246.05177973489</v>
@@ -11558,7 +11568,7 @@
     </row>
     <row r="155">
       <c r="A155" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="B155" s="2" t="n">
         <v>242.944698592225</v>
@@ -11617,7 +11627,7 @@
     </row>
     <row r="156">
       <c r="A156" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="B156" s="2" t="n">
         <v>221.815192021166</v>
@@ -11676,7 +11686,7 @@
     </row>
     <row r="157">
       <c r="A157" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="B157" s="2" t="n">
         <v>190.075015101373</v>
@@ -11735,7 +11745,7 @@
     </row>
     <row r="158">
       <c r="A158" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="B158" s="2" t="n">
         <v>186.084122104724</v>
@@ -11794,7 +11804,7 @@
     </row>
     <row r="159">
       <c r="A159" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="B159" s="2" t="n">
         <v>188.570301111737</v>
@@ -11853,7 +11863,7 @@
     </row>
     <row r="160">
       <c r="A160" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="B160" s="2" t="n">
         <v>223.914839100364</v>
@@ -11912,7 +11922,7 @@
     </row>
     <row r="161">
       <c r="A161" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="B161" s="2" t="n">
         <v>268.561452427047</v>
@@ -11971,7 +11981,7 @@
     </row>
     <row r="162">
       <c r="A162" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="B162" s="2" t="n">
         <v>286.780319612315</v>
@@ -12030,7 +12040,7 @@
     </row>
     <row r="163">
       <c r="A163" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="B163" s="2" t="n">
         <v>273.228701622149</v>
@@ -12089,7 +12099,7 @@
     </row>
     <row r="164">
       <c r="A164" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="B164" s="2" t="n">
         <v>267.618316964556</v>
@@ -12148,7 +12158,7 @@
     </row>
     <row r="165">
       <c r="A165" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="B165" s="2" t="n">
         <v>258.062088650737</v>
@@ -12207,7 +12217,7 @@
     </row>
     <row r="166">
       <c r="A166" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="B166" s="2" t="n">
         <v>258.433764885279</v>
@@ -12266,7 +12276,7 @@
     </row>
     <row r="167">
       <c r="A167" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="B167" s="2" t="n">
         <v>259.854416049084</v>
@@ -12325,7 +12335,7 @@
     </row>
     <row r="168">
       <c r="A168" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="B168" s="2" t="n">
         <v>238.802547979623</v>
@@ -12384,7 +12394,7 @@
     </row>
     <row r="169">
       <c r="A169" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="B169" s="2" t="n">
         <v>205.430496568736</v>
@@ -12443,7 +12453,7 @@
     </row>
     <row r="170">
       <c r="A170" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="B170" s="2" t="n">
         <v>203.521420115062</v>
@@ -12502,7 +12512,7 @@
     </row>
     <row r="171">
       <c r="A171" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="B171" s="2" t="n">
         <v>205.407957919488</v>
@@ -12561,7 +12571,7 @@
     </row>
     <row r="172">
       <c r="A172" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="B172" s="2" t="n">
         <v>238.785921742525</v>
@@ -12620,7 +12630,7 @@
     </row>
     <row r="173">
       <c r="A173" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="B173" s="2" t="n">
         <v>283.935519308077</v>
@@ -12679,7 +12689,7 @@
     </row>
     <row r="174">
       <c r="A174" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="B174" s="2" t="n">
         <v>302.723282832334</v>
@@ -12738,7 +12748,7 @@
     </row>
     <row r="175">
       <c r="A175" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="B175" s="2" t="n">
         <v>287.763792965515</v>
@@ -12797,7 +12807,7 @@
     </row>
     <row r="176">
       <c r="A176" t="s">
-        <v>226</v>
+        <v>228</v>
       </c>
       <c r="B176" s="2" t="n">
         <v>283.322194270445</v>
@@ -12856,7 +12866,7 @@
     </row>
     <row r="177">
       <c r="A177" t="s">
-        <v>227</v>
+        <v>229</v>
       </c>
       <c r="B177" s="2" t="n">
         <v>271.744176727999</v>
@@ -12915,7 +12925,7 @@
     </row>
     <row r="178">
       <c r="A178" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="B178" s="2" t="n">
         <v>264.698398851249</v>
@@ -12974,7 +12984,7 @@
     </row>
     <row r="179">
       <c r="A179" t="s">
-        <v>229</v>
+        <v>231</v>
       </c>
       <c r="B179" s="2" t="n">
         <v>259.005191119666</v>
@@ -13033,7 +13043,7 @@
     </row>
     <row r="180">
       <c r="A180" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
       <c r="B180" s="2" t="n">
         <v>232.86088397523</v>
@@ -13092,7 +13102,7 @@
     </row>
     <row r="181">
       <c r="A181" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="B181" s="2" t="n">
         <v>195.435729497449</v>
@@ -13151,7 +13161,7 @@
     </row>
     <row r="182">
       <c r="A182" t="s">
-        <v>232</v>
+        <v>234</v>
       </c>
       <c r="B182" s="2" t="n">
         <v>187.912132374717</v>
@@ -13210,7 +13220,7 @@
     </row>
     <row r="183">
       <c r="A183" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="B183" s="2" t="n">
         <v>185.75337664486</v>
@@ -13269,7 +13279,7 @@
     </row>
     <row r="184">
       <c r="A184" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="B184" s="2" t="n">
         <v>213.844798658858</v>
@@ -13328,7 +13338,7 @@
     </row>
     <row r="185">
       <c r="A185" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="B185" s="2" t="n">
         <v>250.016227072402</v>
@@ -13387,7 +13397,7 @@
     </row>
     <row r="186">
       <c r="A186" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="B186" s="2" t="n">
         <v>264.767666783786</v>
@@ -13446,7 +13456,7 @@
     </row>
     <row r="187">
       <c r="A187" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="B187" s="2" t="n">
         <v>252.622281044264</v>
@@ -13505,7 +13515,7 @@
     </row>
     <row r="188">
       <c r="A188" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="B188" s="2" t="n">
         <v>250.355597794294</v>
@@ -13564,7 +13574,7 @@
     </row>
     <row r="189">
       <c r="A189" t="s">
-        <v>239</v>
+        <v>241</v>
       </c>
       <c r="B189" s="2" t="n">
         <v>245.426569096129</v>
@@ -13623,7 +13633,7 @@
     </row>
     <row r="190">
       <c r="A190" t="s">
-        <v>240</v>
+        <v>242</v>
       </c>
       <c r="B190" s="2" t="n">
         <v>245.220754344814</v>
@@ -13682,7 +13692,7 @@
     </row>
     <row r="191">
       <c r="A191" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
       <c r="B191" s="2" t="n">
         <v>245.500430319328</v>
@@ -13741,7 +13751,7 @@
     </row>
     <row r="192">
       <c r="A192" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
       <c r="B192" s="2" t="n">
         <v>224.486632404763</v>
@@ -13800,7 +13810,7 @@
     </row>
     <row r="193">
       <c r="A193" t="s">
-        <v>243</v>
+        <v>245</v>
       </c>
       <c r="B193" s="2" t="n">
         <v>191.7922825967</v>
@@ -13859,7 +13869,7 @@
     </row>
     <row r="194">
       <c r="A194" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
       <c r="B194" s="2" t="n">
         <v>192.791062373299</v>
@@ -13918,7 +13928,7 @@
     </row>
     <row r="195">
       <c r="A195" t="s">
-        <v>245</v>
+        <v>247</v>
       </c>
       <c r="B195" s="2" t="n">
         <v>200.676312094232</v>
@@ -13977,7 +13987,7 @@
     </row>
     <row r="196">
       <c r="A196" t="s">
-        <v>246</v>
+        <v>248</v>
       </c>
       <c r="B196" s="2" t="n">
         <v>240.480254531947</v>
@@ -14036,7 +14046,7 @@
     </row>
     <row r="197">
       <c r="A197" t="s">
-        <v>247</v>
+        <v>249</v>
       </c>
       <c r="B197" s="2" t="n">
         <v>289.687566169466</v>
@@ -14095,7 +14105,7 @@
     </row>
     <row r="198">
       <c r="A198" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
       <c r="B198" s="2" t="n">
         <v>308.520351976871</v>
@@ -14154,7 +14164,7 @@
     </row>
     <row r="199">
       <c r="A199" t="s">
-        <v>249</v>
+        <v>251</v>
       </c>
       <c r="B199" s="2" t="n">
         <v>295.337395084573</v>
@@ -14213,7 +14223,7 @@
     </row>
     <row r="200">
       <c r="A200" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
       <c r="B200" s="2" t="n">
         <v>295.284204248692</v>
@@ -14272,7 +14282,7 @@
     </row>
     <row r="201">
       <c r="A201" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="B201" s="2" t="n">
         <v>286.586058426147</v>
@@ -14331,7 +14341,7 @@
     </row>
     <row r="202">
       <c r="A202" t="s">
-        <v>252</v>
+        <v>254</v>
       </c>
       <c r="B202" s="2" t="n">
         <v>280.828839087466</v>
@@ -14390,7 +14400,7 @@
     </row>
     <row r="203">
       <c r="A203" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="B203" s="2" t="n">
         <v>277.038782426195</v>
@@ -14449,7 +14459,7 @@
     </row>
     <row r="204">
       <c r="A204" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
       <c r="B204" s="2" t="n">
         <v>251.269822310689</v>
@@ -14508,7 +14518,7 @@
     </row>
     <row r="205">
       <c r="A205" t="s">
-        <v>255</v>
+        <v>257</v>
       </c>
       <c r="B205" s="2" t="n">
         <v>214.333109108887</v>
@@ -14567,7 +14577,7 @@
     </row>
     <row r="206">
       <c r="A206" t="s">
-        <v>256</v>
+        <v>258</v>
       </c>
       <c r="B206" s="2" t="n">
         <v>211.425159548536</v>
@@ -14626,7 +14636,7 @@
     </row>
     <row r="207">
       <c r="A207" t="s">
-        <v>257</v>
+        <v>259</v>
       </c>
       <c r="B207" s="2" t="n">
         <v>210.502108982888</v>
@@ -14685,7 +14695,7 @@
     </row>
     <row r="208">
       <c r="A208" t="s">
-        <v>258</v>
+        <v>260</v>
       </c>
       <c r="B208" s="2" t="n">
         <v>242.496237561406</v>
@@ -14744,7 +14754,7 @@
     </row>
     <row r="209">
       <c r="A209" t="s">
-        <v>259</v>
+        <v>261</v>
       </c>
       <c r="B209" s="2" t="n">
         <v>288.58421684604</v>
@@ -14803,7 +14813,7 @@
     </row>
     <row r="210">
       <c r="A210" t="s">
-        <v>260</v>
+        <v>262</v>
       </c>
       <c r="B210" s="2" t="n">
         <v>308.889063432899</v>
@@ -14862,7 +14872,7 @@
     </row>
     <row r="211">
       <c r="A211" t="s">
-        <v>261</v>
+        <v>263</v>
       </c>
       <c r="B211" s="2" t="n">
         <v>296.624422031901</v>
@@ -14921,7 +14931,7 @@
     </row>
     <row r="212">
       <c r="A212" t="s">
-        <v>262</v>
+        <v>264</v>
       </c>
       <c r="B212" s="2" t="n">
         <v>293.667443530417</v>
@@ -14980,7 +14990,7 @@
     </row>
     <row r="213">
       <c r="A213" t="s">
-        <v>263</v>
+        <v>265</v>
       </c>
       <c r="B213" s="2" t="n">
         <v>281.66355362494</v>
@@ -15039,7 +15049,7 @@
     </row>
     <row r="214">
       <c r="A214" t="s">
-        <v>264</v>
+        <v>266</v>
       </c>
       <c r="B214" s="2" t="n">
         <v>277.352027692687</v>
@@ -15098,7 +15108,7 @@
     </row>
     <row r="215">
       <c r="A215" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="B215" s="2" t="n">
         <v>276.425037341213</v>
@@ -15157,7 +15167,7 @@
     </row>
     <row r="216">
       <c r="A216" t="s">
-        <v>266</v>
+        <v>268</v>
       </c>
       <c r="B216" s="2" t="n">
         <v>251.942387883981</v>
@@ -15216,7 +15226,7 @@
     </row>
     <row r="217">
       <c r="A217" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
       <c r="B217" s="2" t="n">
         <v>213.821118560682</v>
@@ -15275,7 +15285,7 @@
     </row>
     <row r="218">
       <c r="A218" t="s">
-        <v>268</v>
+        <v>270</v>
       </c>
       <c r="B218" s="2" t="n">
         <v>211.5300495</v>
@@ -15334,7 +15344,7 @@
     </row>
     <row r="219">
       <c r="A219" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
       <c r="B219" s="2" t="n">
         <v>211.8974495</v>
@@ -15393,7 +15403,7 @@
     </row>
     <row r="220">
       <c r="A220" t="s">
-        <v>270</v>
+        <v>272</v>
       </c>
       <c r="B220" s="2" t="n">
         <v>226.426009</v>
@@ -15452,7 +15462,7 @@
     </row>
     <row r="221">
       <c r="A221" t="s">
-        <v>271</v>
+        <v>273</v>
       </c>
       <c r="B221" s="2" t="n">
         <v>235.588409</v>
@@ -15511,7 +15521,7 @@
     </row>
     <row r="222">
       <c r="A222" t="s">
-        <v>272</v>
+        <v>274</v>
       </c>
       <c r="B222" s="2" t="n">
         <v>244.1698535</v>
@@ -15570,7 +15580,7 @@
     </row>
     <row r="223">
       <c r="A223" t="s">
-        <v>273</v>
+        <v>275</v>
       </c>
       <c r="B223" s="2" t="n">
         <v>231.3576035</v>
@@ -15629,7 +15639,7 @@
     </row>
     <row r="224">
       <c r="A224" t="s">
-        <v>274</v>
+        <v>276</v>
       </c>
       <c r="B224" s="2" t="n">
         <v>228.454277</v>
@@ -15688,7 +15698,7 @@
     </row>
     <row r="225">
       <c r="A225" t="s">
-        <v>275</v>
+        <v>277</v>
       </c>
       <c r="B225" s="2" t="n">
         <v>228.995433</v>
@@ -15747,7 +15757,7 @@
     </row>
     <row r="226">
       <c r="A226" t="s">
-        <v>276</v>
+        <v>278</v>
       </c>
       <c r="B226" s="2" t="n">
         <v>228.002157</v>
@@ -15806,7 +15816,7 @@
     </row>
     <row r="227">
       <c r="A227" t="s">
-        <v>277</v>
+        <v>279</v>
       </c>
       <c r="B227" s="2" t="n">
         <v>219.290618</v>
@@ -15865,7 +15875,7 @@
     </row>
     <row r="228">
       <c r="A228" t="s">
-        <v>278</v>
+        <v>280</v>
       </c>
       <c r="B228" s="2" t="n">
         <v>217.82623</v>
@@ -15924,7 +15934,7 @@
     </row>
     <row r="229">
       <c r="A229" t="s">
-        <v>279</v>
+        <v>281</v>
       </c>
       <c r="B229" s="2" t="n">
         <v>201.02397</v>
@@ -15983,7 +15993,7 @@
     </row>
     <row r="230">
       <c r="A230" t="s">
-        <v>280</v>
+        <v>282</v>
       </c>
       <c r="B230" s="2" t="n">
         <v>197.7229065</v>
@@ -16042,7 +16052,7 @@
     </row>
     <row r="231">
       <c r="A231" t="s">
-        <v>281</v>
+        <v>283</v>
       </c>
       <c r="B231" s="2" t="n">
         <v>199.6594105</v>
@@ -16101,7 +16111,7 @@
     </row>
     <row r="232">
       <c r="A232" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="B232" s="2" t="n">
         <v>211.7106645</v>
@@ -16160,7 +16170,7 @@
     </row>
     <row r="233">
       <c r="A233" t="s">
-        <v>283</v>
+        <v>285</v>
       </c>
       <c r="B233" s="2" t="n">
         <v>246.7782865</v>
@@ -16219,7 +16229,7 @@
     </row>
     <row r="234">
       <c r="A234" t="s">
-        <v>284</v>
+        <v>286</v>
       </c>
       <c r="B234" s="2" t="n">
         <v>255.0022115</v>
@@ -16278,7 +16288,7 @@
     </row>
     <row r="235">
       <c r="A235" t="s">
-        <v>285</v>
+        <v>287</v>
       </c>
       <c r="B235" s="2" t="n">
         <v>245.5589415</v>
@@ -16337,7 +16347,7 @@
     </row>
     <row r="236">
       <c r="A236" t="s">
-        <v>286</v>
+        <v>288</v>
       </c>
       <c r="B236" s="2" t="n">
         <v>249.01217</v>
@@ -16396,7 +16406,7 @@
     </row>
     <row r="237">
       <c r="A237" t="s">
-        <v>287</v>
+        <v>289</v>
       </c>
       <c r="B237" s="2" t="n">
         <v>243.263229</v>
@@ -16455,7 +16465,7 @@
     </row>
     <row r="238">
       <c r="A238" t="s">
-        <v>288</v>
+        <v>290</v>
       </c>
       <c r="B238" s="2" t="n">
         <v>241.365337</v>
@@ -16514,7 +16524,7 @@
     </row>
     <row r="239">
       <c r="A239" t="s">
-        <v>289</v>
+        <v>291</v>
       </c>
       <c r="B239" s="2" t="n">
         <v>231.804128</v>
@@ -16573,7 +16583,7 @@
     </row>
     <row r="240">
       <c r="A240" t="s">
-        <v>290</v>
+        <v>292</v>
       </c>
       <c r="B240" s="2" t="n">
         <v>216.647745</v>
@@ -16632,7 +16642,7 @@
     </row>
     <row r="241">
       <c r="A241" t="s">
-        <v>291</v>
+        <v>293</v>
       </c>
       <c r="B241" s="2" t="n">
         <v>196.271098</v>
@@ -16691,7 +16701,7 @@
     </row>
     <row r="242">
       <c r="A242" t="s">
-        <v>292</v>
+        <v>294</v>
       </c>
       <c r="B242" s="2" t="n">
         <v>192.893605</v>
@@ -16750,7 +16760,7 @@
     </row>
     <row r="243">
       <c r="A243" t="s">
-        <v>293</v>
+        <v>295</v>
       </c>
       <c r="B243" s="2" t="n">
         <v>190.429076</v>
@@ -16809,7 +16819,7 @@
     </row>
     <row r="244">
       <c r="A244" t="s">
-        <v>294</v>
+        <v>296</v>
       </c>
       <c r="B244" s="2" t="n">
         <v>212.695477</v>
@@ -16868,7 +16878,7 @@
     </row>
     <row r="245">
       <c r="A245" t="s">
-        <v>295</v>
+        <v>297</v>
       </c>
       <c r="B245" s="2" t="n">
         <v>233.693596</v>
@@ -16927,7 +16937,7 @@
     </row>
     <row r="246">
       <c r="A246" t="s">
-        <v>296</v>
+        <v>298</v>
       </c>
       <c r="B246" s="2" t="n">
         <v>243.219512</v>
@@ -16986,7 +16996,7 @@
     </row>
     <row r="247">
       <c r="A247" t="s">
-        <v>297</v>
+        <v>299</v>
       </c>
       <c r="B247" s="2" t="n">
         <v>244.15752</v>
@@ -17045,7 +17055,7 @@
     </row>
     <row r="248">
       <c r="A248" t="s">
-        <v>298</v>
+        <v>300</v>
       </c>
       <c r="B248" s="2" t="n">
         <v>238.698</v>
@@ -17104,7 +17114,7 @@
     </row>
     <row r="249">
       <c r="A249" t="s">
-        <v>299</v>
+        <v>301</v>
       </c>
       <c r="B249" s="2" t="n">
         <v>230.3679</v>
@@ -17163,7 +17173,7 @@
     </row>
     <row r="250">
       <c r="A250" t="s">
-        <v>300</v>
+        <v>302</v>
       </c>
       <c r="B250" s="2" t="n">
         <v>227.7420205</v>
@@ -17222,7 +17232,7 @@
     </row>
     <row r="251">
       <c r="A251" t="s">
-        <v>301</v>
+        <v>303</v>
       </c>
       <c r="B251" s="2" t="n">
         <v>242.5303445</v>
@@ -17281,7 +17291,7 @@
     </row>
     <row r="252">
       <c r="A252" t="s">
-        <v>302</v>
+        <v>304</v>
       </c>
       <c r="B252" s="2" t="n">
         <v>223.666355</v>
@@ -17340,7 +17350,7 @@
     </row>
     <row r="253">
       <c r="A253" t="s">
-        <v>303</v>
+        <v>305</v>
       </c>
       <c r="B253" s="2" t="n">
         <v>207.479969</v>
@@ -17399,7 +17409,7 @@
     </row>
     <row r="254">
       <c r="A254" t="s">
-        <v>304</v>
+        <v>306</v>
       </c>
       <c r="B254" s="2" t="n">
         <v>189.861485</v>
@@ -17458,7 +17468,7 @@
     </row>
     <row r="255">
       <c r="A255" t="s">
-        <v>305</v>
+        <v>307</v>
       </c>
       <c r="B255" s="2" t="n">
         <v>190.219776</v>
@@ -17517,7 +17527,7 @@
     </row>
     <row r="256">
       <c r="A256" t="s">
-        <v>306</v>
+        <v>308</v>
       </c>
       <c r="B256" s="2" t="n">
         <v>213.5122365</v>
@@ -17576,7 +17586,7 @@
     </row>
     <row r="257">
       <c r="A257" t="s">
-        <v>307</v>
+        <v>309</v>
       </c>
       <c r="B257" s="2" t="n">
         <v>244.2594105</v>
@@ -17635,7 +17645,7 @@
     </row>
     <row r="258">
       <c r="A258" t="s">
-        <v>308</v>
+        <v>310</v>
       </c>
       <c r="B258" s="2" t="n">
         <v>222.3497445</v>
@@ -17694,7 +17704,7 @@
     </row>
     <row r="259">
       <c r="A259" t="s">
-        <v>309</v>
+        <v>311</v>
       </c>
       <c r="B259" s="2" t="n">
         <v>249.3082435</v>
@@ -17753,7 +17763,7 @@
     </row>
     <row r="260">
       <c r="A260" t="s">
-        <v>310</v>
+        <v>312</v>
       </c>
       <c r="B260" s="2" t="n">
         <v>248.7153755</v>
@@ -17812,7 +17822,7 @@
     </row>
     <row r="261">
       <c r="A261" t="s">
-        <v>311</v>
+        <v>313</v>
       </c>
       <c r="B261" s="2" t="n">
         <v>245.0193855</v>
@@ -17871,7 +17881,7 @@
     </row>
     <row r="262">
       <c r="A262" t="s">
-        <v>312</v>
+        <v>314</v>
       </c>
       <c r="B262" s="2" t="n">
         <v>231.5553885</v>
@@ -17930,7 +17940,7 @@
     </row>
     <row r="263">
       <c r="A263" t="s">
-        <v>313</v>
+        <v>315</v>
       </c>
       <c r="B263" s="2" t="n">
         <v>235.6150485</v>
@@ -17989,7 +17999,7 @@
     </row>
     <row r="264">
       <c r="A264" t="s">
-        <v>314</v>
+        <v>316</v>
       </c>
       <c r="B264" s="2" t="n">
         <v>222.911056</v>
@@ -18048,7 +18058,7 @@
     </row>
     <row r="265">
       <c r="A265" t="s">
-        <v>315</v>
+        <v>317</v>
       </c>
       <c r="B265" s="2" t="n">
         <v>205.844239</v>
@@ -18107,7 +18117,7 @@
     </row>
     <row r="266">
       <c r="A266" t="s">
-        <v>316</v>
+        <v>318</v>
       </c>
       <c r="B266" s="2" t="n">
         <v>218.3937465</v>
@@ -18166,7 +18176,7 @@
     </row>
     <row r="267">
       <c r="A267" t="s">
-        <v>317</v>
+        <v>319</v>
       </c>
       <c r="B267" s="2" t="n">
         <v>207.3571735</v>
@@ -18225,7 +18235,7 @@
     </row>
     <row r="268">
       <c r="A268" t="s">
-        <v>318</v>
+        <v>320</v>
       </c>
       <c r="B268" s="2" t="n">
         <v>211.934794</v>
@@ -18284,7 +18294,7 @@
     </row>
     <row r="269">
       <c r="A269" t="s">
-        <v>319</v>
+        <v>321</v>
       </c>
       <c r="B269" s="2" t="n">
         <v>221.378601</v>
@@ -18343,7 +18353,7 @@
     </row>
     <row r="270">
       <c r="A270" t="s">
-        <v>320</v>
+        <v>322</v>
       </c>
       <c r="B270" s="2" t="n">
         <v>221.264134</v>
@@ -18402,7 +18412,7 @@
     </row>
     <row r="271">
       <c r="A271" t="s">
-        <v>321</v>
+        <v>323</v>
       </c>
       <c r="B271" s="2" t="n">
         <v>215.648793</v>
@@ -18461,7 +18471,7 @@
     </row>
     <row r="272">
       <c r="A272" t="s">
-        <v>322</v>
+        <v>324</v>
       </c>
       <c r="B272" s="2" t="n">
         <v>210.378467</v>
@@ -18520,7 +18530,7 @@
     </row>
     <row r="273">
       <c r="A273" t="s">
-        <v>323</v>
+        <v>325</v>
       </c>
       <c r="B273" s="2" t="n">
         <v>217.270382</v>
@@ -18579,7 +18589,7 @@
     </row>
     <row r="274">
       <c r="A274" t="s">
-        <v>324</v>
+        <v>326</v>
       </c>
       <c r="B274" s="2" t="n">
         <v>212.158785</v>
@@ -18638,7 +18648,7 @@
     </row>
     <row r="275">
       <c r="A275" t="s">
-        <v>325</v>
+        <v>327</v>
       </c>
       <c r="B275" s="2" t="n">
         <v>207.728742</v>
@@ -18697,7 +18707,7 @@
     </row>
     <row r="276">
       <c r="A276" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="B276" s="2" t="n">
         <v>211.8548215</v>
@@ -18756,7 +18766,7 @@
     </row>
     <row r="277">
       <c r="A277" t="s">
-        <v>327</v>
+        <v>329</v>
       </c>
       <c r="B277" s="2" t="n">
         <v>198.9981445</v>
@@ -18815,7 +18825,7 @@
     </row>
     <row r="278">
       <c r="A278" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="B278" s="2" t="n">
         <v>207.262923</v>
@@ -18874,7 +18884,7 @@
     </row>
     <row r="279">
       <c r="A279" t="s">
-        <v>329</v>
+        <v>331</v>
       </c>
       <c r="B279" s="2" t="n">
         <v>195.795182</v>
@@ -18933,7 +18943,7 @@
     </row>
     <row r="280">
       <c r="A280" t="s">
-        <v>330</v>
+        <v>332</v>
       </c>
       <c r="B280" s="2" t="n">
         <v>213.3154815</v>
@@ -18992,7 +19002,7 @@
     </row>
     <row r="281">
       <c r="A281" t="s">
-        <v>331</v>
+        <v>333</v>
       </c>
       <c r="B281" s="2" t="n">
         <v>215.7967005</v>
@@ -19051,7 +19061,7 @@
     </row>
     <row r="282">
       <c r="A282" t="s">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="B282" s="2" t="n">
         <v>228.7007085</v>
@@ -19110,7 +19120,7 @@
     </row>
     <row r="283">
       <c r="A283" t="s">
-        <v>333</v>
+        <v>335</v>
       </c>
       <c r="B283" s="2" t="n">
         <v>215.4943715</v>
@@ -19169,7 +19179,7 @@
     </row>
     <row r="284">
       <c r="A284" t="s">
-        <v>334</v>
+        <v>336</v>
       </c>
       <c r="B284" s="2" t="n">
         <v>222.830383</v>
@@ -19228,7 +19238,7 @@
     </row>
     <row r="285">
       <c r="A285" t="s">
-        <v>335</v>
+        <v>337</v>
       </c>
       <c r="B285" s="2" t="n">
         <v>217.021324</v>
@@ -19287,7 +19297,7 @@
     </row>
     <row r="286">
       <c r="A286" t="s">
-        <v>336</v>
+        <v>338</v>
       </c>
       <c r="B286" s="2" t="n">
         <v>205.7906415</v>
@@ -19346,7 +19356,7 @@
     </row>
     <row r="287">
       <c r="A287" t="s">
-        <v>337</v>
+        <v>339</v>
       </c>
       <c r="B287" s="2" t="n">
         <v>217.4511555</v>
@@ -19405,7 +19415,7 @@
     </row>
     <row r="288">
       <c r="A288" t="s">
-        <v>338</v>
+        <v>340</v>
       </c>
       <c r="B288" s="2" t="n">
         <v>212.98443</v>
@@ -19464,7 +19474,7 @@
     </row>
     <row r="289">
       <c r="A289" t="s">
-        <v>339</v>
+        <v>341</v>
       </c>
       <c r="B289" s="2" t="n">
         <v>192.941521</v>
@@ -19523,7 +19533,7 @@
     </row>
     <row r="290">
       <c r="A290" t="s">
-        <v>340</v>
+        <v>342</v>
       </c>
       <c r="B290" s="2" t="n">
         <v>211.9426945</v>
@@ -19582,7 +19592,7 @@
     </row>
     <row r="291">
       <c r="A291" t="s">
-        <v>341</v>
+        <v>343</v>
       </c>
       <c r="B291" s="2" t="n">
         <v>207.4792915</v>
@@ -19641,7 +19651,7 @@
     </row>
     <row r="292">
       <c r="A292" t="s">
-        <v>342</v>
+        <v>344</v>
       </c>
       <c r="B292" s="2" t="n">
         <v>220.4432215</v>
@@ -19700,7 +19710,7 @@
     </row>
     <row r="293">
       <c r="A293" t="s">
-        <v>343</v>
+        <v>345</v>
       </c>
       <c r="B293" s="2" t="n">
         <v>225.1690805</v>
@@ -19759,7 +19769,7 @@
     </row>
     <row r="294">
       <c r="A294" t="s">
-        <v>344</v>
+        <v>346</v>
       </c>
       <c r="B294" s="2" t="n">
         <v>225.213762</v>
@@ -19818,7 +19828,7 @@
     </row>
     <row r="295">
       <c r="A295" t="s">
-        <v>345</v>
+        <v>347</v>
       </c>
       <c r="B295" s="2" t="n">
         <v>214.192024</v>
@@ -19877,7 +19887,7 @@
     </row>
     <row r="296">
       <c r="A296" t="s">
-        <v>346</v>
+        <v>348</v>
       </c>
       <c r="B296" s="2" t="n">
         <v>207.4507435</v>
@@ -19936,7 +19946,7 @@
     </row>
     <row r="297">
       <c r="A297" t="s">
-        <v>347</v>
+        <v>349</v>
       </c>
       <c r="B297" s="2" t="n">
         <v>200.3675575</v>
@@ -19995,7 +20005,7 @@
     </row>
     <row r="298">
       <c r="A298" t="s">
-        <v>348</v>
+        <v>350</v>
       </c>
       <c r="B298" s="2" t="n">
         <v>196.2725365</v>
@@ -20054,7 +20064,7 @@
     </row>
     <row r="299">
       <c r="A299" t="s">
-        <v>349</v>
+        <v>351</v>
       </c>
       <c r="B299" s="2" t="n">
         <v>207.6654335</v>
@@ -20113,7 +20123,7 @@
     </row>
     <row r="300">
       <c r="A300" t="s">
-        <v>350</v>
+        <v>352</v>
       </c>
       <c r="B300" s="2" t="n">
         <v>204.545954</v>
@@ -20172,7 +20182,7 @@
     </row>
     <row r="301">
       <c r="A301" t="s">
-        <v>351</v>
+        <v>353</v>
       </c>
       <c r="B301" s="2" t="n">
         <v>175.216671</v>
@@ -20231,7 +20241,7 @@
     </row>
     <row r="302">
       <c r="A302" t="s">
-        <v>352</v>
+        <v>354</v>
       </c>
       <c r="B302" s="2" t="n">
         <v>192.35973</v>
@@ -20290,7 +20300,7 @@
     </row>
     <row r="303">
       <c r="A303" t="s">
-        <v>353</v>
+        <v>355</v>
       </c>
       <c r="B303" s="2" t="n">
         <v>192.00501</v>
@@ -20349,7 +20359,7 @@
     </row>
     <row r="304">
       <c r="A304" t="s">
-        <v>354</v>
+        <v>356</v>
       </c>
       <c r="B304" s="2" t="n">
         <v>188.7647535</v>
@@ -20408,7 +20418,7 @@
     </row>
     <row r="305">
       <c r="A305" t="s">
-        <v>355</v>
+        <v>357</v>
       </c>
       <c r="B305" s="2" t="n">
         <v>215.0102545</v>
@@ -20467,7 +20477,7 @@
     </row>
     <row r="306">
       <c r="A306" t="s">
-        <v>356</v>
+        <v>358</v>
       </c>
       <c r="B306" s="2" t="n">
         <v>217.606862</v>
@@ -20526,7 +20536,7 @@
     </row>
     <row r="307">
       <c r="A307" t="s">
-        <v>357</v>
+        <v>359</v>
       </c>
       <c r="B307" s="2" t="n">
         <v>209.558405</v>
@@ -20585,7 +20595,7 @@
     </row>
     <row r="308">
       <c r="A308" t="s">
-        <v>358</v>
+        <v>360</v>
       </c>
       <c r="B308" s="2" t="n">
         <v>221.559121</v>
@@ -20644,7 +20654,7 @@
     </row>
     <row r="309">
       <c r="A309" t="s">
-        <v>359</v>
+        <v>361</v>
       </c>
       <c r="B309" s="2" t="n">
         <v>215.719782</v>
@@ -20703,7 +20713,7 @@
     </row>
     <row r="310">
       <c r="A310" t="s">
-        <v>360</v>
+        <v>362</v>
       </c>
       <c r="B310" s="2" t="n">
         <v>197.4669165</v>
@@ -20762,7 +20772,7 @@
     </row>
     <row r="311">
       <c r="A311" t="s">
-        <v>361</v>
+        <v>363</v>
       </c>
       <c r="B311" s="2" t="n">
         <v>217.7495305</v>
@@ -20821,7 +20831,7 @@
     </row>
     <row r="312">
       <c r="A312" t="s">
-        <v>362</v>
+        <v>364</v>
       </c>
       <c r="B312" s="2" t="n">
         <v>207.579178</v>
@@ -20880,7 +20890,7 @@
     </row>
     <row r="313">
       <c r="A313" t="s">
-        <v>363</v>
+        <v>365</v>
       </c>
       <c r="B313" s="2" t="n">
         <v>187.858326</v>
@@ -20939,7 +20949,7 @@
     </row>
     <row r="314">
       <c r="A314" t="s">
-        <v>364</v>
+        <v>366</v>
       </c>
       <c r="B314" s="2" t="n">
         <v>205.3110795</v>
@@ -20998,7 +21008,7 @@
     </row>
     <row r="315">
       <c r="A315" t="s">
-        <v>365</v>
+        <v>367</v>
       </c>
       <c r="B315" s="2" t="n">
         <v>193.0635135</v>
@@ -21057,7 +21067,7 @@
     </row>
     <row r="316">
       <c r="A316" t="s">
-        <v>366</v>
+        <v>368</v>
       </c>
       <c r="B316" s="2" t="n">
         <v>183.7721445</v>
@@ -21116,7 +21126,7 @@
     </row>
     <row r="317">
       <c r="A317" t="s">
-        <v>367</v>
+        <v>369</v>
       </c>
       <c r="B317" s="2" t="n">
         <v>176.1445905</v>
@@ -21175,7 +21185,7 @@
     </row>
     <row r="318">
       <c r="A318" t="s">
-        <v>368</v>
+        <v>370</v>
       </c>
       <c r="B318" s="2" t="n">
         <v>195.4608805</v>
@@ -21234,7 +21244,7 @@
     </row>
     <row r="319">
       <c r="A319" t="s">
-        <v>369</v>
+        <v>371</v>
       </c>
       <c r="B319" s="2" t="n">
         <v>194.4146795</v>
@@ -21293,7 +21303,7 @@
     </row>
     <row r="320">
       <c r="A320" t="s">
-        <v>370</v>
+        <v>372</v>
       </c>
       <c r="B320" s="2" t="n">
         <v>199.682206</v>
@@ -21352,7 +21362,7 @@
     </row>
     <row r="321">
       <c r="A321" t="s">
-        <v>371</v>
+        <v>373</v>
       </c>
       <c r="B321" s="2" t="n">
         <v>203.227869</v>
@@ -21411,7 +21421,7 @@
     </row>
     <row r="322">
       <c r="A322" t="s">
-        <v>372</v>
+        <v>374</v>
       </c>
       <c r="B322" s="2" t="n">
         <v>203.7960685</v>
@@ -21470,7 +21480,7 @@
     </row>
     <row r="323">
       <c r="A323" t="s">
-        <v>373</v>
+        <v>375</v>
       </c>
       <c r="B323" s="2" t="n">
         <v>197.4626355</v>
@@ -21529,7 +21539,7 @@
     </row>
     <row r="324">
       <c r="A324" t="s">
-        <v>374</v>
+        <v>376</v>
       </c>
       <c r="B324" s="2" t="n">
         <v>211.254254</v>
@@ -21588,7 +21598,7 @@
     </row>
     <row r="325">
       <c r="A325" t="s">
-        <v>375</v>
+        <v>377</v>
       </c>
       <c r="B325" s="2" t="n">
         <v>166.343135</v>
@@ -21647,7 +21657,7 @@
     </row>
     <row r="326">
       <c r="A326" t="s">
-        <v>376</v>
+        <v>378</v>
       </c>
       <c r="B326" s="2" t="n">
         <v>232.34734</v>
@@ -21706,7 +21716,7 @@
     </row>
     <row r="327">
       <c r="A327" t="s">
-        <v>377</v>
+        <v>379</v>
       </c>
       <c r="B327" s="2" t="n">
         <v>231.797712</v>
@@ -21765,7 +21775,7 @@
     </row>
     <row r="328">
       <c r="A328" t="s">
-        <v>378</v>
+        <v>380</v>
       </c>
       <c r="B328" s="2" t="n">
         <v>258.5618155</v>
@@ -21824,7 +21834,7 @@
     </row>
     <row r="329">
       <c r="A329" t="s">
-        <v>379</v>
+        <v>381</v>
       </c>
       <c r="B329" s="2" t="n">
         <v>249.4538125</v>
@@ -21883,7 +21893,7 @@
     </row>
     <row r="330">
       <c r="A330" t="s">
-        <v>380</v>
+        <v>382</v>
       </c>
       <c r="B330" s="2" t="n">
         <v>238.968523</v>
@@ -21942,7 +21952,7 @@
     </row>
     <row r="331">
       <c r="A331" t="s">
-        <v>381</v>
+        <v>383</v>
       </c>
       <c r="B331" s="2" t="n">
         <v>241.40421</v>
@@ -22001,7 +22011,7 @@
     </row>
     <row r="332">
       <c r="A332" t="s">
-        <v>382</v>
+        <v>384</v>
       </c>
       <c r="B332" s="2" t="n">
         <v>255.1779355</v>
@@ -22060,7 +22070,7 @@
     </row>
     <row r="333">
       <c r="A333" t="s">
-        <v>383</v>
+        <v>385</v>
       </c>
       <c r="B333" s="2" t="n">
         <v>245.6048305</v>
@@ -22119,7 +22129,7 @@
     </row>
     <row r="334">
       <c r="A334" t="s">
-        <v>384</v>
+        <v>386</v>
       </c>
       <c r="B334" s="2" t="n">
         <v>237.9903375</v>
@@ -22178,7 +22188,7 @@
     </row>
     <row r="335">
       <c r="A335" t="s">
-        <v>385</v>
+        <v>387</v>
       </c>
       <c r="B335" s="2" t="n">
         <v>240.6311285</v>
@@ -22237,7 +22247,7 @@
     </row>
     <row r="336">
       <c r="A336" t="s">
-        <v>386</v>
+        <v>388</v>
       </c>
       <c r="B336" s="2" t="n">
         <v>246.0594505</v>
@@ -22296,7 +22306,7 @@
     </row>
     <row r="337">
       <c r="A337" t="s">
-        <v>387</v>
+        <v>389</v>
       </c>
       <c r="B337" s="2" t="n">
         <v>236.4014155</v>
@@ -22355,7 +22365,7 @@
     </row>
     <row r="338">
       <c r="A338" t="s">
-        <v>388</v>
+        <v>390</v>
       </c>
       <c r="B338" s="2" t="n">
         <v>238.337836</v>
@@ -22414,7 +22424,7 @@
     </row>
     <row r="339">
       <c r="A339" t="s">
-        <v>389</v>
+        <v>391</v>
       </c>
       <c r="B339" s="2" t="n">
         <v>247.690316</v>
@@ -22473,7 +22483,7 @@
     </row>
     <row r="340">
       <c r="A340" t="s">
-        <v>390</v>
+        <v>392</v>
       </c>
       <c r="B340" s="2" t="n">
         <v>255.936923</v>
@@ -22532,7 +22542,7 @@
     </row>
     <row r="341">
       <c r="A341" t="s">
-        <v>391</v>
+        <v>393</v>
       </c>
       <c r="B341" s="2" t="n">
         <v>272.768513</v>
@@ -22591,7 +22601,7 @@
     </row>
     <row r="342">
       <c r="A342" t="s">
-        <v>392</v>
+        <v>394</v>
       </c>
       <c r="B342" s="2" t="n">
         <v>280.5362735</v>
@@ -22650,7 +22660,7 @@
     </row>
     <row r="343">
       <c r="A343" t="s">
-        <v>393</v>
+        <v>395</v>
       </c>
       <c r="B343" s="2" t="n">
         <v>268.2429235</v>
@@ -22709,7 +22719,7 @@
     </row>
     <row r="344">
       <c r="A344" t="s">
-        <v>394</v>
+        <v>396</v>
       </c>
       <c r="B344" s="2" t="n">
         <v>262.1086635</v>
@@ -22768,7 +22778,7 @@
     </row>
     <row r="345">
       <c r="A345" t="s">
-        <v>395</v>
+        <v>397</v>
       </c>
       <c r="B345" s="2" t="n">
         <v>250.8028145</v>
@@ -22827,7 +22837,7 @@
     </row>
     <row r="346">
       <c r="A346" t="s">
-        <v>396</v>
+        <v>398</v>
       </c>
       <c r="B346" s="2" t="n">
         <v>257.8711825</v>
@@ -22886,7 +22896,7 @@
     </row>
     <row r="347">
       <c r="A347" t="s">
-        <v>397</v>
+        <v>399</v>
       </c>
       <c r="B347" s="2" t="n">
         <v>250.9312345</v>
@@ -22945,7 +22955,7 @@
     </row>
     <row r="348">
       <c r="A348" t="s">
-        <v>398</v>
+        <v>400</v>
       </c>
       <c r="B348" s="2" t="n">
         <v>255.8549095</v>
@@ -23004,7 +23014,7 @@
     </row>
     <row r="349">
       <c r="A349" t="s">
-        <v>399</v>
+        <v>401</v>
       </c>
       <c r="B349" s="2" t="n">
         <v>241.8363505</v>
@@ -23063,7 +23073,7 @@
     </row>
     <row r="350">
       <c r="A350" t="s">
-        <v>400</v>
+        <v>402</v>
       </c>
       <c r="B350" s="2" t="n">
         <v>234.082402</v>
@@ -23122,7 +23132,7 @@
     </row>
     <row r="351">
       <c r="A351" t="s">
-        <v>401</v>
+        <v>403</v>
       </c>
       <c r="B351" s="2" t="n">
         <v>219.334761</v>
@@ -23181,7 +23191,7 @@
     </row>
     <row r="352">
       <c r="A352" t="s">
-        <v>402</v>
+        <v>404</v>
       </c>
       <c r="B352" s="2" t="n">
         <v>258.733914</v>
@@ -23240,7 +23250,7 @@
     </row>
     <row r="353">
       <c r="A353" t="s">
-        <v>403</v>
+        <v>405</v>
       </c>
       <c r="B353" s="2" t="n">
         <v>242.842761</v>
@@ -23299,7 +23309,7 @@
     </row>
     <row r="354">
       <c r="A354" t="s">
-        <v>404</v>
+        <v>406</v>
       </c>
       <c r="B354" s="2" t="n">
         <v>258.056234</v>
@@ -23358,7 +23368,7 @@
     </row>
     <row r="355">
       <c r="A355" t="s">
-        <v>405</v>
+        <v>407</v>
       </c>
       <c r="B355" s="2" t="n">
         <v>258.086762</v>
@@ -23417,7 +23427,7 @@
     </row>
     <row r="356">
       <c r="A356" t="s">
-        <v>406</v>
+        <v>408</v>
       </c>
       <c r="B356" s="2" t="n">
         <v>251.0049775</v>
@@ -23476,7 +23486,7 @@
     </row>
     <row r="357">
       <c r="A357" t="s">
-        <v>407</v>
+        <v>409</v>
       </c>
       <c r="B357" s="2" t="n">
         <v>246.0227095</v>
@@ -23535,7 +23545,7 @@
     </row>
     <row r="358">
       <c r="A358" t="s">
-        <v>408</v>
+        <v>410</v>
       </c>
       <c r="B358" s="2" t="n">
         <v>225.7465225</v>
@@ -23594,7 +23604,7 @@
     </row>
     <row r="359">
       <c r="A359" t="s">
-        <v>409</v>
+        <v>411</v>
       </c>
       <c r="B359" s="2" t="n">
         <v>224.6182285</v>
@@ -23653,7 +23663,7 @@
     </row>
     <row r="360">
       <c r="A360" t="s">
-        <v>410</v>
+        <v>412</v>
       </c>
       <c r="B360" s="2" t="n">
         <v>223.0257775</v>
@@ -23712,7 +23722,7 @@
     </row>
     <row r="361">
       <c r="A361" t="s">
-        <v>411</v>
+        <v>413</v>
       </c>
       <c r="B361" s="2" t="n">
         <v>218.8956025</v>
@@ -23771,7 +23781,7 @@
     </row>
     <row r="362">
       <c r="A362" t="s">
-        <v>412</v>
+        <v>414</v>
       </c>
       <c r="B362" s="2" t="n">
         <v>228.7973315</v>
@@ -23830,7 +23840,7 @@
     </row>
     <row r="363">
       <c r="A363" t="s">
-        <v>413</v>
+        <v>415</v>
       </c>
       <c r="B363" s="2" t="n">
         <v>235.1951405</v>
@@ -23889,7 +23899,7 @@
     </row>
     <row r="364">
       <c r="A364" t="s">
-        <v>414</v>
+        <v>416</v>
       </c>
       <c r="B364" s="2" t="n">
         <v>247.6812475</v>
@@ -23948,7 +23958,7 @@
     </row>
     <row r="365">
       <c r="A365" t="s">
-        <v>415</v>
+        <v>417</v>
       </c>
       <c r="B365" s="2" t="n">
         <v>245.0149465</v>
@@ -24007,7 +24017,7 @@
     </row>
     <row r="366">
       <c r="A366" t="s">
-        <v>416</v>
+        <v>418</v>
       </c>
       <c r="B366" s="2" t="n">
         <v>249.703611</v>
@@ -24066,7 +24076,7 @@
     </row>
     <row r="367">
       <c r="A367" t="s">
-        <v>417</v>
+        <v>419</v>
       </c>
       <c r="B367" s="2" t="n">
         <v>230.680739</v>
@@ -24125,7 +24135,7 @@
     </row>
     <row r="368">
       <c r="A368" t="s">
-        <v>418</v>
+        <v>420</v>
       </c>
       <c r="B368" s="2" t="n">
         <v>246.1225485</v>
@@ -24184,7 +24194,7 @@
     </row>
     <row r="369">
       <c r="A369" t="s">
-        <v>419</v>
+        <v>421</v>
       </c>
       <c r="B369" s="2" t="n">
         <v>235.8910035</v>
@@ -24243,7 +24253,7 @@
     </row>
     <row r="370">
       <c r="A370" t="s">
-        <v>420</v>
+        <v>422</v>
       </c>
       <c r="B370" s="2" t="n">
         <v>248.7751265</v>
@@ -24302,7 +24312,7 @@
     </row>
     <row r="371">
       <c r="A371" t="s">
-        <v>421</v>
+        <v>423</v>
       </c>
       <c r="B371" s="2" t="n">
         <v>260.1399005</v>
@@ -24361,7 +24371,7 @@
     </row>
     <row r="372">
       <c r="A372" t="s">
-        <v>422</v>
+        <v>424</v>
       </c>
       <c r="B372" s="2" t="n">
         <v>239.2236185</v>
@@ -24420,7 +24430,7 @@
     </row>
     <row r="373">
       <c r="A373" t="s">
-        <v>423</v>
+        <v>425</v>
       </c>
       <c r="B373" s="2" t="n">
         <v>229.6022875</v>
@@ -24479,7 +24489,7 @@
     </row>
     <row r="374">
       <c r="A374" t="s">
-        <v>424</v>
+        <v>426</v>
       </c>
       <c r="B374" s="2" t="n">
         <v>239.42136924</v>
@@ -24538,7 +24548,7 @@
     </row>
     <row r="375">
       <c r="A375" t="s">
-        <v>425</v>
+        <v>427</v>
       </c>
       <c r="B375" s="2" t="n">
         <v>237.72979551</v>
@@ -24597,7 +24607,7 @@
     </row>
     <row r="376">
       <c r="A376" t="s">
-        <v>426</v>
+        <v>428</v>
       </c>
       <c r="B376" s="2" t="n">
         <v>236.58174443</v>
@@ -24656,7 +24666,7 @@
     </row>
     <row r="377">
       <c r="A377" t="s">
-        <v>427</v>
+        <v>429</v>
       </c>
       <c r="B377" s="2" t="n">
         <v>234.00800894</v>
@@ -24715,7 +24725,7 @@
     </row>
     <row r="378">
       <c r="A378" t="s">
-        <v>428</v>
+        <v>430</v>
       </c>
       <c r="B378" s="2" t="n">
         <v>245.51211575</v>
@@ -24774,7 +24784,7 @@
     </row>
     <row r="379">
       <c r="A379" t="s">
-        <v>429</v>
+        <v>431</v>
       </c>
       <c r="B379" s="2" t="n">
         <v>228.51356787</v>
@@ -24833,7 +24843,7 @@
     </row>
     <row r="380">
       <c r="A380" t="s">
-        <v>430</v>
+        <v>432</v>
       </c>
       <c r="B380" s="2" t="n">
         <v>211.0047266</v>
@@ -24892,7 +24902,7 @@
     </row>
     <row r="381">
       <c r="A381" t="s">
-        <v>431</v>
+        <v>433</v>
       </c>
       <c r="B381" s="2" t="n">
         <v>244.44648976</v>
@@ -24951,7 +24961,7 @@
     </row>
     <row r="382">
       <c r="A382" t="s">
-        <v>432</v>
+        <v>434</v>
       </c>
       <c r="B382" s="2" t="n">
         <v>239.88042486</v>
@@ -25010,7 +25020,7 @@
     </row>
     <row r="383">
       <c r="A383" t="s">
-        <v>433</v>
+        <v>435</v>
       </c>
       <c r="B383" s="2" t="n">
         <v>239.93725186</v>
@@ -25069,7 +25079,7 @@
     </row>
     <row r="384">
       <c r="A384" t="s">
-        <v>434</v>
+        <v>436</v>
       </c>
       <c r="B384" s="2" t="n">
         <v>227.71951947</v>
@@ -25128,7 +25138,7 @@
     </row>
     <row r="385">
       <c r="A385" t="s">
-        <v>435</v>
+        <v>437</v>
       </c>
       <c r="B385" s="2" t="n">
         <v>229.04942849</v>
@@ -25187,7 +25197,7 @@
     </row>
     <row r="386">
       <c r="A386" t="s">
-        <v>436</v>
+        <v>438</v>
       </c>
       <c r="B386" s="2" t="n">
         <v>223.55917359</v>
@@ -25246,7 +25256,7 @@
     </row>
     <row r="387">
       <c r="A387" t="s">
-        <v>437</v>
+        <v>439</v>
       </c>
       <c r="B387" s="2" t="n">
         <v>199.31492533</v>
@@ -25305,7 +25315,7 @@
     </row>
     <row r="388">
       <c r="A388" t="s">
-        <v>438</v>
+        <v>440</v>
       </c>
       <c r="B388" s="2" t="n">
         <v>244.18779529</v>
@@ -25364,7 +25374,7 @@
     </row>
     <row r="389">
       <c r="A389" t="s">
-        <v>439</v>
+        <v>441</v>
       </c>
       <c r="B389" s="2" t="n">
         <v>235.81625292</v>
@@ -25423,7 +25433,7 @@
     </row>
     <row r="390">
       <c r="A390" t="s">
-        <v>440</v>
+        <v>442</v>
       </c>
       <c r="B390" s="2"/>
       <c r="C390" s="3" t="n">
@@ -25456,7 +25466,7 @@
     </row>
     <row r="391">
       <c r="A391" t="s">
-        <v>441</v>
+        <v>443</v>
       </c>
       <c r="B391" s="2"/>
       <c r="C391" s="3" t="n">
@@ -25489,7 +25499,7 @@
     </row>
     <row r="392">
       <c r="A392" t="s">
-        <v>442</v>
+        <v>444</v>
       </c>
       <c r="B392" s="2"/>
       <c r="C392" s="3" t="n">
@@ -25522,7 +25532,7 @@
     </row>
     <row r="393">
       <c r="A393" t="s">
-        <v>443</v>
+        <v>445</v>
       </c>
       <c r="B393" s="2"/>
       <c r="C393" s="3" t="n">
@@ -25555,7 +25565,7 @@
     </row>
     <row r="394">
       <c r="A394" t="s">
-        <v>444</v>
+        <v>446</v>
       </c>
       <c r="B394" s="2"/>
       <c r="C394" s="3" t="n">
@@ -25588,7 +25598,7 @@
     </row>
     <row r="395">
       <c r="A395" t="s">
-        <v>445</v>
+        <v>447</v>
       </c>
       <c r="B395" s="2"/>
       <c r="C395" s="3" t="n">
@@ -25621,7 +25631,7 @@
     </row>
     <row r="396">
       <c r="A396" t="s">
-        <v>446</v>
+        <v>448</v>
       </c>
       <c r="B396" s="2"/>
       <c r="C396" s="3" t="n">
@@ -25654,7 +25664,7 @@
     </row>
     <row r="397">
       <c r="A397" t="s">
-        <v>447</v>
+        <v>449</v>
       </c>
       <c r="B397" s="2"/>
       <c r="C397" s="3" t="n">
@@ -25687,7 +25697,7 @@
     </row>
     <row r="398">
       <c r="A398" t="s">
-        <v>448</v>
+        <v>450</v>
       </c>
       <c r="B398" s="2"/>
       <c r="C398" s="3" t="n">
@@ -25720,7 +25730,7 @@
     </row>
     <row r="399">
       <c r="A399" t="s">
-        <v>449</v>
+        <v>451</v>
       </c>
       <c r="B399" s="2"/>
       <c r="C399" s="3" t="n">
@@ -25753,7 +25763,7 @@
     </row>
     <row r="400">
       <c r="A400" t="s">
-        <v>450</v>
+        <v>452</v>
       </c>
       <c r="B400" s="2"/>
       <c r="C400" s="3" t="n">
@@ -25786,7 +25796,7 @@
     </row>
     <row r="401">
       <c r="A401" t="s">
-        <v>451</v>
+        <v>453</v>
       </c>
       <c r="B401" s="2"/>
       <c r="C401" s="3" t="n">
@@ -25819,7 +25829,7 @@
     </row>
     <row r="402">
       <c r="A402" t="s">
-        <v>452</v>
+        <v>454</v>
       </c>
       <c r="B402" s="2"/>
       <c r="C402" s="3"/>
@@ -25842,7 +25852,7 @@
     </row>
     <row r="403">
       <c r="A403" t="s">
-        <v>453</v>
+        <v>455</v>
       </c>
       <c r="B403" s="2"/>
       <c r="C403" s="3"/>
@@ -25865,7 +25875,7 @@
     </row>
     <row r="404">
       <c r="A404" t="s">
-        <v>454</v>
+        <v>456</v>
       </c>
       <c r="B404" s="2"/>
       <c r="C404" s="3"/>
@@ -25888,7 +25898,7 @@
     </row>
     <row r="405">
       <c r="A405" t="s">
-        <v>455</v>
+        <v>457</v>
       </c>
       <c r="B405" s="2"/>
       <c r="C405" s="3"/>
@@ -25911,7 +25921,7 @@
     </row>
     <row r="406">
       <c r="A406" t="s">
-        <v>456</v>
+        <v>458</v>
       </c>
       <c r="B406" s="2"/>
       <c r="C406" s="3"/>
@@ -25934,7 +25944,7 @@
     </row>
     <row r="407">
       <c r="A407" t="s">
-        <v>457</v>
+        <v>459</v>
       </c>
       <c r="B407" s="2"/>
       <c r="C407" s="3"/>
@@ -25957,7 +25967,7 @@
     </row>
     <row r="408">
       <c r="A408" t="s">
-        <v>458</v>
+        <v>460</v>
       </c>
       <c r="B408" s="2"/>
       <c r="C408" s="3"/>
@@ -25980,7 +25990,7 @@
     </row>
     <row r="409">
       <c r="A409" t="s">
-        <v>459</v>
+        <v>461</v>
       </c>
       <c r="B409" s="2"/>
       <c r="C409" s="3"/>
@@ -26003,7 +26013,7 @@
     </row>
     <row r="410">
       <c r="A410" t="s">
-        <v>460</v>
+        <v>462</v>
       </c>
       <c r="B410" s="2"/>
       <c r="C410" s="3"/>
@@ -26026,7 +26036,7 @@
     </row>
     <row r="411">
       <c r="A411" t="s">
-        <v>461</v>
+        <v>463</v>
       </c>
       <c r="B411" s="2"/>
       <c r="C411" s="3"/>
@@ -26049,7 +26059,7 @@
     </row>
     <row r="412">
       <c r="A412" t="s">
-        <v>462</v>
+        <v>464</v>
       </c>
       <c r="B412" s="2"/>
       <c r="C412" s="3"/>
@@ -26072,7 +26082,7 @@
     </row>
     <row r="413">
       <c r="A413" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
       <c r="B413" s="2"/>
       <c r="C413" s="3"/>
@@ -26095,7 +26105,7 @@
     </row>
     <row r="414">
       <c r="A414" t="s">
-        <v>464</v>
+        <v>466</v>
       </c>
       <c r="B414" s="2"/>
       <c r="C414" s="3"/>
@@ -26118,7 +26128,7 @@
     </row>
     <row r="415">
       <c r="A415" t="s">
-        <v>465</v>
+        <v>467</v>
       </c>
       <c r="B415" s="2"/>
       <c r="C415" s="3"/>
@@ -26141,7 +26151,7 @@
     </row>
     <row r="416">
       <c r="A416" t="s">
-        <v>466</v>
+        <v>468</v>
       </c>
       <c r="B416" s="2"/>
       <c r="C416" s="3"/>
@@ -26164,7 +26174,7 @@
     </row>
     <row r="417">
       <c r="A417" t="s">
-        <v>467</v>
+        <v>469</v>
       </c>
       <c r="B417" s="2"/>
       <c r="C417" s="3"/>
@@ -26187,7 +26197,7 @@
     </row>
     <row r="418">
       <c r="A418" t="s">
-        <v>468</v>
+        <v>470</v>
       </c>
       <c r="B418" s="2"/>
       <c r="C418" s="3"/>
@@ -26210,7 +26220,7 @@
     </row>
     <row r="419">
       <c r="A419" t="s">
-        <v>469</v>
+        <v>471</v>
       </c>
       <c r="B419" s="2"/>
       <c r="C419" s="3"/>
@@ -26233,7 +26243,7 @@
     </row>
     <row r="420">
       <c r="A420" t="s">
-        <v>470</v>
+        <v>472</v>
       </c>
       <c r="B420" s="2"/>
       <c r="C420" s="3"/>
@@ -26256,7 +26266,7 @@
     </row>
     <row r="421">
       <c r="A421" t="s">
-        <v>471</v>
+        <v>473</v>
       </c>
       <c r="B421" s="2"/>
       <c r="C421" s="3"/>
@@ -26279,7 +26289,7 @@
     </row>
     <row r="422">
       <c r="A422" t="s">
-        <v>472</v>
+        <v>474</v>
       </c>
       <c r="B422" s="2"/>
       <c r="C422" s="3"/>
@@ -26302,7 +26312,7 @@
     </row>
     <row r="423">
       <c r="A423" t="s">
-        <v>473</v>
+        <v>475</v>
       </c>
       <c r="B423" s="2"/>
       <c r="C423" s="3"/>
@@ -26325,7 +26335,7 @@
     </row>
     <row r="424">
       <c r="A424" t="s">
-        <v>474</v>
+        <v>476</v>
       </c>
       <c r="B424" s="2"/>
       <c r="C424" s="3"/>
@@ -26348,7 +26358,7 @@
     </row>
     <row r="425">
       <c r="A425" t="s">
-        <v>475</v>
+        <v>477</v>
       </c>
       <c r="B425" s="2"/>
       <c r="C425" s="3"/>
@@ -26371,7 +26381,7 @@
     </row>
     <row r="426">
       <c r="A426" t="s">
-        <v>476</v>
+        <v>478</v>
       </c>
       <c r="B426" s="2"/>
       <c r="C426" s="3"/>
@@ -26394,7 +26404,7 @@
     </row>
     <row r="427">
       <c r="A427" t="s">
-        <v>477</v>
+        <v>479</v>
       </c>
       <c r="B427" s="2"/>
       <c r="C427" s="3"/>
@@ -26417,7 +26427,7 @@
     </row>
     <row r="428">
       <c r="A428" t="s">
-        <v>478</v>
+        <v>480</v>
       </c>
       <c r="B428" s="2"/>
       <c r="C428" s="3"/>
@@ -26440,7 +26450,7 @@
     </row>
     <row r="429">
       <c r="A429" t="s">
-        <v>479</v>
+        <v>481</v>
       </c>
       <c r="B429" s="2"/>
       <c r="C429" s="3"/>
@@ -26463,7 +26473,7 @@
     </row>
     <row r="430">
       <c r="A430" t="s">
-        <v>480</v>
+        <v>482</v>
       </c>
       <c r="B430" s="2"/>
       <c r="C430" s="3"/>
@@ -26486,7 +26496,7 @@
     </row>
     <row r="431">
       <c r="A431" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
       <c r="B431" s="2"/>
       <c r="C431" s="3"/>
@@ -26509,7 +26519,7 @@
     </row>
     <row r="432">
       <c r="A432" t="s">
-        <v>482</v>
+        <v>484</v>
       </c>
       <c r="B432" s="2"/>
       <c r="C432" s="3"/>
@@ -26532,7 +26542,7 @@
     </row>
     <row r="433">
       <c r="A433" t="s">
-        <v>483</v>
+        <v>485</v>
       </c>
       <c r="B433" s="2"/>
       <c r="C433" s="3"/>
@@ -26555,7 +26565,7 @@
     </row>
     <row r="434">
       <c r="A434" t="s">
-        <v>484</v>
+        <v>486</v>
       </c>
       <c r="B434" s="2"/>
       <c r="C434" s="3"/>
@@ -26578,7 +26588,7 @@
     </row>
     <row r="435">
       <c r="A435" t="s">
-        <v>485</v>
+        <v>487</v>
       </c>
       <c r="B435" s="2"/>
       <c r="C435" s="3"/>
@@ -26601,7 +26611,7 @@
     </row>
     <row r="436">
       <c r="A436" t="s">
-        <v>486</v>
+        <v>488</v>
       </c>
       <c r="B436" s="2"/>
       <c r="C436" s="3"/>
@@ -26624,7 +26634,7 @@
     </row>
     <row r="437">
       <c r="A437" t="s">
-        <v>487</v>
+        <v>489</v>
       </c>
       <c r="B437" s="2"/>
       <c r="C437" s="3"/>
@@ -26647,7 +26657,7 @@
     </row>
     <row r="438">
       <c r="A438" t="s">
-        <v>488</v>
+        <v>490</v>
       </c>
       <c r="B438" s="2"/>
       <c r="C438" s="3"/>
@@ -26670,7 +26680,7 @@
     </row>
     <row r="439">
       <c r="A439" t="s">
-        <v>489</v>
+        <v>491</v>
       </c>
       <c r="B439" s="2"/>
       <c r="C439" s="3"/>
@@ -26693,7 +26703,7 @@
     </row>
     <row r="440">
       <c r="A440" t="s">
-        <v>490</v>
+        <v>492</v>
       </c>
       <c r="B440" s="2"/>
       <c r="C440" s="3"/>
@@ -26716,7 +26726,7 @@
     </row>
     <row r="441">
       <c r="A441" t="s">
-        <v>491</v>
+        <v>493</v>
       </c>
       <c r="B441" s="2"/>
       <c r="C441" s="3"/>
@@ -26739,7 +26749,7 @@
     </row>
     <row r="442">
       <c r="A442" t="s">
-        <v>492</v>
+        <v>494</v>
       </c>
       <c r="B442" s="2"/>
       <c r="C442" s="3"/>
@@ -26762,7 +26772,7 @@
     </row>
     <row r="443">
       <c r="A443" t="s">
-        <v>493</v>
+        <v>495</v>
       </c>
       <c r="B443" s="2"/>
       <c r="C443" s="3"/>
@@ -26785,7 +26795,7 @@
     </row>
     <row r="444">
       <c r="A444" t="s">
-        <v>494</v>
+        <v>496</v>
       </c>
       <c r="B444" s="2"/>
       <c r="C444" s="3"/>
@@ -26808,7 +26818,7 @@
     </row>
     <row r="445">
       <c r="A445" t="s">
-        <v>495</v>
+        <v>497</v>
       </c>
       <c r="B445" s="2"/>
       <c r="C445" s="3"/>
@@ -26842,97 +26852,97 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>496</v>
+        <v>498</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>497</v>
+        <v>499</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>498</v>
+        <v>500</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>499</v>
+        <v>501</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>500</v>
+        <v>502</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>501</v>
+        <v>503</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>502</v>
+        <v>504</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>503</v>
+        <v>505</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>504</v>
+        <v>506</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>505</v>
+        <v>507</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>506</v>
+        <v>508</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>507</v>
+        <v>509</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>508</v>
+        <v>510</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>509</v>
+        <v>511</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>510</v>
+        <v>512</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>511</v>
+        <v>513</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>512</v>
+        <v>514</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>513</v>
+        <v>515</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>514</v>
+        <v>516</v>
       </c>
     </row>
   </sheetData>
@@ -26956,7 +26966,7 @@
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>515</v>
+        <v>517</v>
       </c>
       <c r="B2" s="1"/>
     </row>
@@ -26966,160 +26976,160 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>516</v>
+        <v>518</v>
       </c>
       <c r="B4" s="1"/>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>517</v>
+        <v>519</v>
       </c>
       <c r="B5" s="1" t="n">
-        <v>0.0978575452575677</v>
+        <v>0.0980921257379144</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>518</v>
+        <v>520</v>
       </c>
       <c r="B6" s="1" t="n">
-        <v>0.127047032380892</v>
+        <v>0.126632428187349</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>519</v>
+        <v>521</v>
       </c>
       <c r="B7" s="1" t="n">
-        <v>0.165288503880143</v>
+        <v>0.163228654443303</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>520</v>
+        <v>522</v>
       </c>
       <c r="B8" s="1" t="n">
-        <v>0.218486051842877</v>
+        <v>0.21614769417722</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>521</v>
+        <v>523</v>
       </c>
       <c r="B9" s="1" t="n">
-        <v>0.285059447334508</v>
+        <v>0.283736815297369</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>522</v>
+        <v>524</v>
       </c>
       <c r="B10" s="1" t="n">
-        <v>0.360380975680041</v>
+        <v>0.358487029231923</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>523</v>
+        <v>525</v>
       </c>
       <c r="B11" s="1" t="n">
-        <v>0.443403525737214</v>
+        <v>0.44025771644677</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>524</v>
+        <v>526</v>
       </c>
       <c r="B12" s="1" t="n">
-        <v>0.503539915434965</v>
+        <v>0.501933156219224</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>525</v>
+        <v>527</v>
       </c>
       <c r="B13" s="1" t="n">
-        <v>0.52098946735509</v>
+        <v>0.521586057839713</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>526</v>
+        <v>528</v>
       </c>
       <c r="B14" s="1" t="n">
-        <v>0.493180293132542</v>
+        <v>0.494487808856228</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>527</v>
+        <v>529</v>
       </c>
       <c r="B15" s="1" t="n">
-        <v>0.407982976059349</v>
+        <v>0.409760749491849</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>528</v>
+        <v>530</v>
       </c>
       <c r="B16" s="1" t="n">
-        <v>0.307815574335169</v>
+        <v>0.30949070976312</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>529</v>
+        <v>531</v>
       </c>
       <c r="B17" s="1" t="n">
-        <v>0.246405326157374</v>
+        <v>0.24885760706515</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>530</v>
+        <v>532</v>
       </c>
       <c r="B18" s="1" t="n">
-        <v>0.190294080499725</v>
+        <v>0.193037112533873</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>531</v>
+        <v>533</v>
       </c>
       <c r="B19" s="1" t="n">
-        <v>0.112224883707372</v>
+        <v>0.114218256723769</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>532</v>
+        <v>534</v>
       </c>
       <c r="B20" s="1" t="n">
-        <v>0.02322442118176</v>
+        <v>0.023791174836451</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="s">
-        <v>533</v>
+        <v>535</v>
       </c>
       <c r="B21" s="1" t="n">
-        <v>-0.0618455187713708</v>
+        <v>-0.0623205680268032</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="s">
-        <v>534</v>
+        <v>536</v>
       </c>
       <c r="B22" s="1" t="n">
-        <v>-0.117514023650424</v>
+        <v>-0.117141657290668</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="s">
-        <v>535</v>
+        <v>537</v>
       </c>
       <c r="B23" s="1" t="n">
-        <v>-0.150976288588822</v>
+        <v>-0.149262769348846</v>
       </c>
     </row>
     <row r="24">

</xml_diff>